<commit_message>
feat: harden FormulaWitness evaluation and repair
</commit_message>
<xml_diff>
--- a/artifacts/submission/m10/repaired.xlsx
+++ b/artifacts/submission/m10/repaired.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Cover" sheetId="1" r:id="Rba8a792bf82c4fa9"/>
-    <sheet name="RebateCalc" sheetId="2" r:id="Rf4a98c3f2a6a4291"/>
-    <sheet name="Checks" sheetId="3" r:id="Rf5139066236f4bc9"/>
-    <sheet name="Counterexamples" sheetId="4" r:id="rIdFormulaWitness4"/>
-    <sheet name="FormulaWitness_Report" sheetId="5" r:id="rIdFormulaWitness5"/>
+    <sheet name="Cover" sheetId="1" r:id="Rdcf202c8ed674ea0"/>
+    <sheet name="RebateCalc" sheetId="2" r:id="R28809b2a6eed4473"/>
+    <sheet name="TierSchedule" sheetId="3" r:id="R22f7e560b35e49be"/>
+    <sheet name="Checks" sheetId="4" r:id="Rf0aa090b72bf40f1"/>
+    <sheet name="Counterexamples" sheetId="5" r:id="rIdFormulaWitness5"/>
+    <sheet name="FormulaWitness_Report" sheetId="6" r:id="rIdFormulaWitness6"/>
   </sheets>
 </workbook>
 </file>
@@ -17,15 +18,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="6">
+  <x:numFmts count="7">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="$#,##0.00;[Red]($#,##0.00);-"/>
     <x:numFmt numFmtId="202" formatCode="0.0%;[Red](0.0%);-"/>
     <x:numFmt numFmtId="203" formatCode="0"/>
     <x:numFmt numFmtId="204" formatCode="0.0%"/>
     <x:numFmt numFmtId="205" formatCode="0.00x"/>
+    <x:numFmt numFmtId="206" formatCode="$#,##0.00"/>
   </x:numFmts>
-  <x:fonts count="11">
+  <x:fonts count="12">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -78,6 +80,12 @@
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FF475569"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="17"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
@@ -135,7 +143,7 @@
       </x:patternFill>
     </x:fill>
   </x:fills>
-  <x:borders count="13">
+  <x:borders count="18">
     <x:border/>
     <x:border>
       <x:left style="thin">
@@ -227,11 +235,69 @@
         <x:color rgb="FFAAB6C7"/>
       </x:bottom>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB8C4D6"/>
+      </x:top>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="75">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -321,13 +387,30 @@
     <x:xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="206" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center"/>
     </x:xf>
   </x:cellXfs>
@@ -807,7 +890,7 @@
         <v>SLA multiplier</v>
       </c>
       <c r="Q5" s="34" t="str">
-        <v>Tenure multiplier</v>
+        <v>Effective proration</v>
       </c>
       <c r="R5" s="34" t="str">
         <v>Adjusted rebate</v>
@@ -862,7 +945,7 @@
         <v>90</v>
       </c>
       <c r="N6" s="50" t="n">
-        <f>IF(L6&lt;100000,0,IF(L6&lt;250000,0.02,IF(L6&lt;500000,0.03,0.04)))</f>
+        <f>LOOKUP(L6,TierSchedule!A5:A8,TierSchedule!B5:B8)</f>
         <v>0.03</v>
       </c>
       <c r="O6" s="48" t="n">
@@ -873,7 +956,7 @@
         <f>IF(AND(J6&gt;=1,K6&lt;&gt;"Y"),0,IF(AND(H6&lt;0.95,I6&gt;0.02),0.6,IF(OR(H6&lt;0.95,I6&gt;0.02),0.75,1)))</f>
       </c>
       <c r="Q6" s="51" t="n">
-        <f>IF(M6&lt;90,0.5,1)</f>
+        <f>MIN(1,M6/MAX(1,C6-B6+1))</f>
         <v>1</v>
       </c>
       <c r="R6" s="48" t="n">
@@ -944,6 +1027,108 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
+    <x:col min="1" max="1" width="24" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="56" t="str">
+        <x:v>Controlled ordered tier lookup</x:v>
+      </x:c>
+      <x:c r="B1" s="56"/>
+      <x:c r="C1" s="56"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="56"/>
+      <x:c r="B2" s="56"/>
+      <x:c r="C2" s="56"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="23" t="str">
+        <x:v>Lower bound (inclusive)</x:v>
+      </x:c>
+      <x:c r="B4" s="23" t="str">
+        <x:v>Rate</x:v>
+      </x:c>
+      <x:c r="C4" s="23" t="str">
+        <x:v>Upper-bound behavior</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="64" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="B5" s="67" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="C5" s="58" t="str">
+        <x:v>below 100,000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="65" t="n">
+        <x:v>100000</x:v>
+      </x:c>
+      <x:c r="B6" s="68" t="n">
+        <x:v>0.02</x:v>
+      </x:c>
+      <x:c r="C6" s="61" t="str">
+        <x:v>below 250,000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="65" t="n">
+        <x:v>250000</x:v>
+      </x:c>
+      <x:c r="B7" s="68" t="n">
+        <x:v>0.03</x:v>
+      </x:c>
+      <x:c r="C7" s="61" t="str">
+        <x:v>below 500,000</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="66" t="n">
+        <x:v>500000</x:v>
+      </x:c>
+      <x:c r="B8" s="69" t="n">
+        <x:v>0.04</x:v>
+      </x:c>
+      <x:c r="C8" s="63" t="str">
+        <x:v>no upper bound</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="54" t="str">
+        <x:v>RebateCalc!N6 uses Excel LOOKUP against A5:B8. M03–M05 shift a narrow interval at each inclusive lower bound.</x:v>
+      </x:c>
+      <x:c r="B10" s="54"/>
+      <x:c r="C10" s="54"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="54"/>
+      <x:c r="B11" s="54"/>
+      <x:c r="C11" s="54"/>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="54"/>
+      <x:c r="B12" s="54"/>
+      <x:c r="C12" s="54"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:C2"/>
+    <x:mergeCell ref="A10:C12"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
     <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
@@ -953,22 +1138,22 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1">
-      <x:c r="A1" s="55" t="str">
+      <x:c r="A1" s="70" t="str">
         <x:v>Model Controls</x:v>
       </x:c>
-      <x:c r="B1" s="55"/>
-      <x:c r="C1" s="55"/>
-      <x:c r="D1" s="55"/>
-      <x:c r="E1" s="55"/>
-      <x:c r="F1" s="55"/>
+      <x:c r="B1" s="70"/>
+      <x:c r="C1" s="70"/>
+      <x:c r="D1" s="70"/>
+      <x:c r="E1" s="70"/>
+      <x:c r="F1" s="70"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="55"/>
-      <x:c r="B2" s="55"/>
-      <x:c r="C2" s="55"/>
-      <x:c r="D2" s="55"/>
-      <x:c r="E2" s="55"/>
-      <x:c r="F2" s="55"/>
+      <x:c r="A2" s="70"/>
+      <x:c r="B2" s="70"/>
+      <x:c r="C2" s="70"/>
+      <x:c r="D2" s="70"/>
+      <x:c r="E2" s="70"/>
+      <x:c r="F2" s="70"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="23" t="str">
@@ -1083,17 +1268,17 @@
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="56" t="str">
+      <x:c r="A10" s="71" t="str">
         <x:v>MODEL STATUS</x:v>
       </x:c>
-      <x:c r="B10" s="56"/>
-      <x:c r="C10" s="56"/>
-      <x:c r="D10" s="56"/>
-      <x:c r="E10" s="59" t="str">
+      <x:c r="B10" s="71"/>
+      <x:c r="C10" s="71"/>
+      <x:c r="D10" s="71"/>
+      <x:c r="E10" s="74" t="str">
         <x:f>IF(COUNTIF(E5:E8,"FAIL")=0,"PASS","FAIL")</x:f>
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="F10" s="59"/>
+      <x:c r="F10" s="74"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1105,7 +1290,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1882,7 +2067,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>tenure_90</t>
+          <t>proration_full_period</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1924,7 +2109,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>tenure_89</t>
+          <t>proration_89_of_90_days</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1949,12 +2134,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>S6=3750; T6=PAYABLE</t>
+          <t>S6=7416.67; T6=PAYABLE</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>S6=3750; T6=PAYABLE</t>
+          <t>S6=7416.67; T6=PAYABLE</t>
         </is>
       </c>
     </row>
@@ -2004,7 +2189,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -2031,7 +2216,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>advanced-9e4a2e37c326</t>
+          <t>advanced-f569ca78b557</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2252,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>5beb61724aad4368960ad215205b1043f0afccb7b0931115cb2ca1a9c47f51af</t>
+          <t>d3485903dc07d662e1373ac59993b19ec54ff733ae2de411450acefea8af8762</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2264,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>945ee0c6b6147843dcc20818b1a2a2d5a677b270d75a9c1d605bab92d4b45819</t>
+          <t>72f8b8dfbf2104d453678f0c258031f1b7cadf0890e19af4727e163324f79b84</t>
         </is>
       </c>
     </row>
@@ -2091,7 +2276,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>32f946f03cc9595533a9d4e9d0292a9b2a174b76a5cc7efcb55850487cec751e</t>
+          <t/>
         </is>
       </c>
     </row>

</xml_diff>